<commit_message>
Update ANFORA validation workbooks
Refresh the mid-validation data collection and innovator indicators workbooks with the latest revisions.
</commit_message>
<xml_diff>
--- a/Innovator Indicators Review 2026-10-21/ANFORA_Innovator_Indicators_Updated_2026-10-21_Rev3.xlsx
+++ b/Innovator Indicators Review 2026-10-21/ANFORA_Innovator_Indicators_Updated_2026-10-21_Rev3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lasith/Downloads/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jmvev\Desktop\Mid Validation - Anfora\Innovator Indicators Review 2026-10-21\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{161440A7-B9ED-5A45-B664-6A37DBCD4F20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27162324-8A04-4D73-AC5F-A2787984638B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{787A48DC-CF7E-1645-832C-CD73A594925B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{787A48DC-CF7E-1645-832C-CD73A594925B}"/>
   </bookViews>
   <sheets>
     <sheet name="D05-ANFORA" sheetId="5" r:id="rId1"/>
@@ -27,16 +27,17 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="135">
   <si>
     <t>Innovator Name</t>
   </si>
@@ -227,9 +228,6 @@
     <t>Guadalquivir basin WEI+ baseline to be retrieved from Eurostat/CHG at project start (M1). Andalucía is classified by the EEA as a water-scarce region with recurrent structural water stress.</t>
   </si>
   <si>
-    <t>Contextual indicator. ANFORA contributes indirectly by enabling a 10–15% reduction of water footprint among early adopters (KPI18), linked to RDD1 and the Cross-cutting Priority of Climate Change Adaptation. Data sources: Eurostat, Confederación Hidrográfica del Guadalquivir (CHG), AEMET, Junta de Andalucía.</t>
-  </si>
-  <si>
     <t>Citizen involvement in environmental education activities (Total)</t>
   </si>
   <si>
@@ -269,9 +267,6 @@
     <t>0 (no ANFORA-led training activities prior to M13).</t>
   </si>
   <si>
-    <t>Target aligned with KPI17 (50 users trained) via 5–10 workshops of max. 15 participants (Activity 3.2, M13–M16) complemented by on-demand video tutorials. Engages youth &lt;30, adults &gt;55, long-term unemployed, farmers and agri-food industry.</t>
-  </si>
-  <si>
     <t>Number of new jobs in green sector (Total)</t>
   </si>
   <si>
@@ -296,9 +291,6 @@
     <t>0 new jobs directly attributable to ANFORA at project start (M1).</t>
   </si>
   <si>
-    <t>The project mobilises 5.45 Person-Months across the Evenor-Tech team (Dra. María Anaya Romero —coordinator—, Dr. Félix González Peñaloza, Dr. Francisco J. Blanco Velázquez, MSc Javier Bravo García, MSc Fernando Alonso Martín). Target: consolidate at least 1 FTE opportunity in digital green services. Contributes to RDD2 and to the Social Justice &amp; Inclusion cross-cutting priority.</t>
-  </si>
-  <si>
     <t>Total number of participants in citizen engagement activities (workshops, co-creation sessions, awareness campaigns).</t>
   </si>
   <si>
@@ -314,9 +306,6 @@
     <t>0 registered users at project start (platform goes live in Phase 3, M13).</t>
   </si>
   <si>
-    <t>Target aligned with KPI16 (100 registered users within 2 months of launch, Activity 3.1). Complemented by KPI8 (50 stakeholder interviews, Activity 1.1) during Phase 1 co-design. Pilot sites in Lucena: Coop. Lucena, Agrocor, Almazaras D.O. Montilla-Moriles, Cervecería Cruz Blanca, Bodeguita del Casino, Precocinados La Alacena, etc.</t>
-  </si>
-  <si>
     <t>Energy consumption of irrigation systems (kWh/ha)</t>
   </si>
   <si>
@@ -347,24 +336,12 @@
     <t>Baseline per crop/farm to be measured in Phase 1 (M3–M6), subject to a formal collaboration agreement with irrigation communities in the Guadalquivir basin.</t>
   </si>
   <si>
-    <t>Innovator indicator — not included in the original KREI list. Addresses the water–energy–food nexus and contributes to RDD3 (Energy Transition and Climate Neutrality). Data captured from smart meters and farm logs of participating Lucena agri-cooperatives.</t>
-  </si>
-  <si>
     <t>User interaction data from digital platforms</t>
   </si>
   <si>
     <t>Complements KPIs 16 &amp; 17 (registered and trained users), offering deeper insights into platform adoption and behavioural change.</t>
   </si>
   <si>
-    <t>Platform usage logs</t>
-  </si>
-  <si>
-    <t>Currently: backend `morgan` request logs + `winston` application logs. Web analytics (Hotjar, Google Analytics, Sentry) to be integrated in Phase 2/3.</t>
-  </si>
-  <si>
-    <t>Server / App</t>
-  </si>
-  <si>
     <t># users, sessions</t>
   </si>
   <si>
@@ -374,27 +351,15 @@
     <t>0 users / sessions before public launch (M13).</t>
   </si>
   <si>
-    <t>Innovator indicator — not in the KREI list. Complements KPI15 (&lt;10 critical incidents, Activity 2.2) and KPI16 (100 registered users). Web-analytics tools (Hotjar, Google Analytics, Sentry) and front-end instrumentation are still to be deployed; current data comes from `morgan` / `winston` server-side logs on api.anfora.evenor-tech.com. Once available, this indicator will also feed the AI module that personalises methodology selection (WFN / ISO 14046 / LCA / recipe / diet) — itself planned for Phase 3.</t>
-  </si>
-  <si>
     <t>Water saved through behavioural change (litres or %)</t>
   </si>
   <si>
     <t>Difference between baseline water footprint and adjusted diet/recipe/product choices simulated in ANFORA.</t>
   </si>
   <si>
-    <t>Platform calculations</t>
-  </si>
-  <si>
-    <t>App / Dashboard</t>
-  </si>
-  <si>
     <t>Per user action</t>
   </si>
   <si>
-    <t>Server (AI model)</t>
-  </si>
-  <si>
     <t>Litres / %</t>
   </si>
   <si>
@@ -404,27 +369,15 @@
     <t>Initial water footprint per user/recipe/diet, calculated automatically by the platform on first use (reference scenario).</t>
   </si>
   <si>
-    <t>Innovator indicator — not in the KREI list. Direct operationalisation of KPI18 (10–15% water footprint reduction, Activity 4.1) and complements KPI19 (average satisfaction ≥4/5). Implemented by comparing the baseline calculation against alternatives proposed by the AI recommender and user-adjusted recipes ("recipe-to-table" digital twin).</t>
-  </si>
-  <si>
     <t>EWI: Low User Engagement Alert</t>
   </si>
   <si>
     <t>Early Warning Indicator that triggers an alert when satisfaction scores in pilot tests fall below 80% or when the average satisfaction score drops under 4/5, enabling corrective actions on usability, content or training.</t>
   </si>
   <si>
-    <t>Post-test satisfaction surveys (dedicated feedback module to be implemented in Phase 2 — currently only a free-text contact-form `feedback` template exists in the backend).</t>
-  </si>
-  <si>
-    <t>Survey tool (to be selected) + future platform feedback module. Front-end monitoring (Sentry / Hotjar) planned for Phase 2/3.</t>
-  </si>
-  <si>
     <t>Periodic (per pilot / per event)</t>
   </si>
   <si>
-    <t>Survey tool + platform feedback module (planned, Phase 2/3). Front-end monitoring (Sentry / Hotjar) not yet integrated.</t>
-  </si>
-  <si>
     <t>% satisfaction / score (1–5)</t>
   </si>
   <si>
@@ -437,27 +390,15 @@
     <t>No alerts before pilot tests (Activity 2.1 starts in M7).</t>
   </si>
   <si>
-    <t>Early Warning Indicator suggested by the mentoring team. Linked to KPI14 (80–90% satisfaction) and KPI19 (≥4/5). Mitigates the "User Adoption Resistance" risk identified in Section 5.5 of the Technical Proposal.</t>
-  </si>
-  <si>
     <t>EWI: Demographic Imbalance Alert</t>
   </si>
   <si>
     <t>Early Warning Indicator that monitors whether ANFORA effectively reaches vulnerable groups — people under 30, people over 55 and the long-term unemployed — to safeguard social inclusion in line with the Cross-cutting Priority.</t>
   </si>
   <si>
-    <t>Registration form (self-declared age group &amp; employment status — fields to be added to the `User` model in Phase 2; currently the schema only stores name / email / password / lastLogin / profileImage) and training attendance lists.</t>
-  </si>
-  <si>
-    <t>Platform registration + workshop logs</t>
-  </si>
-  <si>
     <t>Periodic (per event / cohort)</t>
   </si>
   <si>
-    <t>Platform database (MongoDB) + attendance sheets</t>
-  </si>
-  <si>
     <t>% per target group</t>
   </si>
   <si>
@@ -470,14 +411,80 @@
     <t>No data before platform launch (M13). Preliminary outreach to potential user sites defined in Activity 1.1 (Lucena cooperatives, markets, hospitality, cafeterias).</t>
   </si>
   <si>
-    <t>Early Warning Indicator suggested by the mentoring team. Supports the Social Justice and Inclusion cross-cutting priority and informs the training strategy under Activity 3.2 (KPI17: 50 users trained).</t>
+    <t>Evenor-Tech S.L.U.</t>
+  </si>
+  <si>
+    <t>Declared result: 0 persons trained, 1 March–31 August 2026. Evenor-Tech confirms that no training activities with participants took place. This is an internal responsible-party declaration, not a signed certificate or independently verified attendance count. The 48-person statement concerns September–October and is excluded. Source: Evenor-Tech confirmation, 21 October 2026. Hybrid (AMT + API) was accepted on 2 September 2026. Per-indicator routing and technical integration remain pending; auto_accept is unassigned (blank).</t>
+  </si>
+  <si>
+    <t>Not measured for March–August 2026. Evenor-Tech confirms no irrigation electricity-consumption measurements per hectare. Water-footprint calculations cannot supply kWh/ha. Required: dated electricity readings and irrigated area for the same farms/crops and seasonal or annual baseline. Source: Evenor-Tech confirmation, 21 October 2026. Hybrid (AMT + API) was accepted on 2 September 2026. Per-indicator routing and technical integration remain pending; auto_accept is unassigned (blank).</t>
+  </si>
+  <si>
+    <t>Three retained PostHog CSVs and Evenor-Tech confirmation (21 October 2026); separate read-only MongoDB aggregates.</t>
+  </si>
+  <si>
+    <t>Check exported daily values and dates. Responsible-party confirmation identifies metric aggregation and internal tests; coverage and external-user attribution remain unverified.</t>
+  </si>
+  <si>
+    <t>ANFORA backend, MongoDB and PostHog. No RURACTIVE indicator feed verified.</t>
+  </si>
+  <si>
+    <t>Matched baseline and follow-up scenarios; no validated longitudinal dataset available.</t>
+  </si>
+  <si>
+    <t>Comparable scenario analysis with consistent sources, quantities and servings.</t>
+  </si>
+  <si>
+    <t>Recipe footprint calculations; no verified AI recommender or behavioural-savings feed.</t>
+  </si>
+  <si>
+    <t>Not measured for March–August 2026. ANFORA supports water-footprint simulations, but no dated valid baseline/alternative scenario pairs are verified. Global versus Andalusian reference values do not establish supermarket versus local-market origin. Comparable sources, quantities and servings are required before reporting litres or percentage savings. Source: retained model/data review and Evenor-Tech confirmation, 21 October 2026. Hybrid (AMT + API) was accepted on 2 September 2026. Per-indicator routing and technical integration remain pending; auto_accept is unassigned (blank).</t>
+  </si>
+  <si>
+    <t>Evenor-Tech confirms no numerical satisfaction survey in March-August 2026.</t>
+  </si>
+  <si>
+    <t>No numerical cohort available; satisfaction/alert not assessable, not zero or FALSE.</t>
+  </si>
+  <si>
+    <t>No validated numerical survey dataset or automated alert result available.</t>
+  </si>
+  <si>
+    <t>Not assessable for March–August 2026. Evenor-Tech confirms that no numerical satisfaction surveys were conducted. Neither satisfaction percentage/mean score nor the alert state can be calculated. Missing survey data do not mean a zero score or a FALSE alert. The official &lt;80% or &lt;4/5 threshold is unchanged. Source: Evenor-Tech confirmation, 21 October 2026. Hybrid (AMT + API) was accepted on 2 September 2026. Per-indicator routing and technical integration remain pending; auto_accept is unassigned (blank).</t>
+  </si>
+  <si>
+    <t>Consent-based age-group and employment declarations plus dated attendance records; dataset unavailable.</t>
+  </si>
+  <si>
+    <t>Eligible group counts and cohort denominator required; no shares computed.</t>
+  </si>
+  <si>
+    <t>Current User schema has no age-group or employment-status fields.</t>
+  </si>
+  <si>
+    <t>Not assessable for March–August 2026. Evenor-Tech confirms insufficient demographic data. Group shares and the imbalance alert cannot be calculated without eligible group counts and a defined cohort denominator. Missing data do not establish 0% representation or a FALSE alert. Source: Evenor-Tech confirmation, 21 October 2026. Hybrid (AMT + API) was accepted on 2 September 2026. Per-indicator routing and technical integration remain pending; auto_accept is unassigned (blank).</t>
+  </si>
+  <si>
+    <t>Not measured for 1 March–31 August 2026. No matched territorial WEI+ observation and baseline are available for the reporting scope. Municipal 2024 water volumes provide context, not WEI+ or attributable ANFORA impact. Source: retained official water-source review. Hybrid (AMT + API) was accepted on 2 September 2026. Per-indicator routing and technical integration remain pending; auto_accept is unassigned (blank).</t>
+  </si>
+  <si>
+    <t>Declared result: 0 new jobs attributable to ANFORA in March–August 2026, confirmed internally by Evenor-Tech on 21 October. No signed HR certification is held. This six-month declaration does not establish the annual result. Hybrid (AMT + API) was accepted on 2 September 2026. Per-indicator routing and technical integration remain pending; auto_accept is unassigned (blank).</t>
+  </si>
+  <si>
+    <t>Declared result: 0 eligible citizen-engagement participants in March–August 2026. Evenor-Tech confirms that the 5 August presentation to Vera/BALAM and Lucena City Council representatives was institutional coordination, not training or an open public citizen activity. Municipal dissemination agreed at that meeting has not materialised. The participant measure and the 100-registered-user target are distinct. Sources: 5 August meeting record and Evenor-Tech confirmation, 21 October; no signed eligible-attendance reconciliation is held. Hybrid (AMT + API) was accepted on 2 September 2026. Per-indicator routing and technical integration remain pending; auto_accept is unassigned (blank).</t>
+  </si>
+  <si>
+    <t>1 March–31 August 2026: external users/sessions are not verified. Three PostHog CSVs show activity only on 31 August: 1 identity, 4 sessions with Pageview and 39 pageviews, as identified by the project lead, who confirms they were his own internal tests. CSVs omit query settings; full-period capture coverage is unproven. Do not infer zero external visits. Two anonymous MongoDB calculations remain separately unclassified. Sources: three retained PostHog exports and Evenor-Tech confirmation, 21 October. Hybrid (AMT + API) agreed 2 September; per-code routing, technical integration and auto_accept remain pending (blank).
+Post-monitoring developments (September–October 2026)
+Excluded from the official period. Read-only MongoDB snapshot: 21 October 2026, 12:55 CEST (Europe/Madrid). Order: accounts / calculations / saved recipes / menus. September: 0 / 3 / 1 / 0; October to the snapshot: 28 / 55 / 27 / 3; historical totals: 33 / 60 / 28 / 3.
+Of October’s 28 accounts, 27 dated 5 October are declared by the project lead to be ADA ITS students’ personal registrations. Sources: MongoDB.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="8">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -771,7 +778,7 @@
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1118,21 +1125,22 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:AB16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19.6640625" style="2" customWidth="1"/>
     <col min="2" max="2" width="46.6640625" style="2" customWidth="1"/>
-    <col min="3" max="5" width="11" style="2"/>
+    <col min="3" max="3" width="15.77734375" style="2" customWidth="1"/>
+    <col min="4" max="5" width="11" style="2"/>
     <col min="6" max="6" width="46.6640625" style="2" customWidth="1"/>
     <col min="7" max="14" width="19.6640625" style="2" customWidth="1"/>
-    <col min="15" max="15" width="44.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="44.44140625" style="2" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="20" style="2" customWidth="1"/>
-    <col min="17" max="17" width="73.1640625" style="2" customWidth="1"/>
-    <col min="18" max="18" width="28.1640625" style="2" customWidth="1"/>
+    <col min="17" max="17" width="73.109375" style="2" customWidth="1"/>
+    <col min="18" max="18" width="28.109375" style="2" customWidth="1"/>
     <col min="19" max="16384" width="11" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:28" ht="15.75">
       <c r="A1"/>
       <c r="B1"/>
       <c r="C1"/>
@@ -1162,7 +1170,7 @@
       <c r="AA1" s="1"/>
       <c r="AB1" s="1"/>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:28" ht="15.75">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -1196,14 +1204,12 @@
       <c r="AA2" s="1"/>
       <c r="AB2" s="1"/>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:28" ht="15.75">
       <c r="A3" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Evenor-Tech S.L.U.</t>
-        </is>
+      <c r="B3" s="29" t="s">
+        <v>113</v>
       </c>
       <c r="C3"/>
       <c r="D3"/>
@@ -1232,7 +1238,7 @@
       <c r="AA3" s="1"/>
       <c r="AB3" s="1"/>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:28" ht="15.75">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1266,7 +1272,7 @@
       <c r="AA4" s="1"/>
       <c r="AB4" s="1"/>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:28" ht="15.75">
       <c r="A5"/>
       <c r="B5"/>
       <c r="C5"/>
@@ -1298,7 +1304,7 @@
       <c r="AA5" s="1"/>
       <c r="AB5" s="1"/>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:28" ht="15.75">
       <c r="A6"/>
       <c r="B6"/>
       <c r="C6"/>
@@ -1328,7 +1334,7 @@
       <c r="AA6" s="1"/>
       <c r="AB6" s="1"/>
     </row>
-    <row r="7" spans="1:28" ht="48" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:28" ht="45">
       <c r="A7" s="5" t="s">
         <v>3</v>
       </c>
@@ -1394,7 +1400,7 @@
       <c r="AA7" s="1"/>
       <c r="AB7" s="1"/>
     </row>
-    <row r="8" spans="1:28" s="4" customFormat="1" ht="170.0" x14ac:dyDescent="0.2" customHeight="1">
+    <row r="8" spans="1:28" s="4" customFormat="1" ht="170.1" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>32</v>
       </c>
@@ -1443,90 +1449,86 @@
       <c r="P8" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="Q8" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not measured for 1 March–31 August 2026. No matched territorial WEI+ observation and baseline are available for the reporting scope. Municipal 2024 water volumes provide context, not WEI+ or attributable ANFORA impact. Lasith must clarify the official ratio/target mapping. Source: retained official water-source review. Hybrid (AMT + API) was accepted on 2 September 2026. Per-indicator routing and technical integration remain pending; auto_accept is unassigned (blank).</t>
-        </is>
+      <c r="Q8" s="12" t="s">
+        <v>131</v>
       </c>
       <c r="R8" s="30"/>
     </row>
-    <row r="9" spans="1:28" s="4" customFormat="1" ht="86.4000015258789" x14ac:dyDescent="0.2" customHeight="1">
+    <row r="9" spans="1:28" s="4" customFormat="1" ht="121.5" customHeight="1">
       <c r="A9" s="15" t="s">
         <v>32</v>
       </c>
       <c r="B9" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="D9" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="E9" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="E9" s="16" t="s">
+      <c r="F9" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="F9" s="16" t="s">
+      <c r="G9" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="G9" s="16" t="s">
+      <c r="H9" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="H9" s="16" t="s">
+      <c r="I9" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="I9" s="16" t="s">
+      <c r="J9" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="J9" s="16" t="s">
+      <c r="K9" s="16" t="s">
         <v>61</v>
-      </c>
-      <c r="K9" s="16" t="s">
-        <v>62</v>
       </c>
       <c r="L9" s="16" t="s">
         <v>20</v>
       </c>
       <c r="M9" s="16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="N9" s="17" t="s">
         <v>49</v>
       </c>
       <c r="O9" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="P9" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="P9" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q9" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Declared result: 0 persons trained, 1 March–31 August 2026. Evenor-Tech confirms that no training activities with participants took place. This is an internal responsible-party declaration, not a signed certificate or independently verified attendance count. The 48-person statement concerns September–October and is excluded. Source: Evenor-Tech confirmation, 21 October 2026. Hybrid (AMT + API) was accepted on 2 September 2026. Per-indicator routing and technical integration remain pending; auto_accept is unassigned (blank).</t>
-        </is>
+      <c r="Q9" s="16" t="s">
+        <v>114</v>
       </c>
       <c r="R9" s="30"/>
     </row>
-    <row r="10" spans="1:28" s="4" customFormat="1" ht="86.4000015258789" x14ac:dyDescent="0.2" customHeight="1">
+    <row r="10" spans="1:28" s="4" customFormat="1" ht="114" customHeight="1">
       <c r="A10" s="15" t="s">
         <v>32</v>
       </c>
       <c r="B10" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="D10" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="E10" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="F10" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="D10" s="16" t="s">
+      <c r="G10" s="16" t="s">
         <v>69</v>
-      </c>
-      <c r="E10" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="F10" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="G10" s="16" t="s">
-        <v>71</v>
       </c>
       <c r="H10" s="16" t="s">
         <v>44</v>
@@ -1538,7 +1540,7 @@
         <v>46</v>
       </c>
       <c r="K10" s="16" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="L10" s="16" t="s">
         <v>20</v>
@@ -1550,19 +1552,17 @@
         <v>49</v>
       </c>
       <c r="O10" s="18" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="P10" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="Q10" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Declared result: 0 new jobs attributable to ANFORA in March–August 2026, confirmed internally by Evenor-Tech on 21 October. No signed HR certification is held. This six-month declaration does not establish the annual result. The official annual frequency, # jobs unit and FTE target are unchanged; annual boundaries and jobs/FTE interpretation require Lasith’s confirmation. Hybrid (AMT + API) was accepted on 2 September 2026. Per-indicator routing and technical integration remain pending; auto_accept is unassigned (blank).</t>
-        </is>
+        <v>72</v>
+      </c>
+      <c r="Q10" s="16" t="s">
+        <v>132</v>
       </c>
       <c r="R10" s="30"/>
     </row>
-    <row r="11" spans="1:28" s="4" customFormat="1" ht="129.60000610351562" x14ac:dyDescent="0.2" customHeight="1">
+    <row r="11" spans="1:28" s="4" customFormat="1" ht="158.25" customHeight="1">
       <c r="A11" s="15" t="s">
         <v>32</v>
       </c>
@@ -1579,51 +1579,49 @@
         <v>29</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="H11" s="16" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="I11" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="J11" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="J11" s="16" t="s">
+      <c r="K11" s="16" t="s">
         <v>61</v>
-      </c>
-      <c r="K11" s="16" t="s">
-        <v>62</v>
       </c>
       <c r="L11" s="16" t="s">
         <v>20</v>
       </c>
       <c r="M11" s="16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="N11" s="17" t="s">
         <v>49</v>
       </c>
       <c r="O11" s="18" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="P11" s="16" t="s">
-        <v>80</v>
-      </c>
-      <c r="Q11" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Declared result: 0 eligible citizen-engagement participants in March–August 2026, subject to Lasith’s acceptance of activity eligibility. Evenor-Tech confirms that the 5 August presentation to Vera/BALAM and Lucena City Council representatives was institutional coordination, not training or an open public citizen activity. Municipal dissemination agreed at that meeting has not materialised. The participant measure and the 100-registered-user target are distinct. Sources: 5 August meeting record and Evenor-Tech confirmation, 21 October; no signed eligible-attendance reconciliation is held. Hybrid (AMT + API) was accepted on 2 September 2026. Per-indicator routing and technical integration remain pending; auto_accept is unassigned (blank).</t>
-        </is>
+        <v>77</v>
+      </c>
+      <c r="Q11" s="16" t="s">
+        <v>133</v>
       </c>
       <c r="R11" s="30"/>
     </row>
-    <row r="12" spans="1:28" s="4" customFormat="1" ht="153.0" x14ac:dyDescent="0.2" customHeight="1">
+    <row r="12" spans="1:28" s="4" customFormat="1" ht="153" customHeight="1">
       <c r="A12" s="19" t="s">
         <v>19</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C12" s="28" t="s">
         <v>30</v>
@@ -1631,51 +1629,49 @@
       <c r="D12" s="27"/>
       <c r="E12" s="27"/>
       <c r="F12" s="21" t="s">
+        <v>79</v>
+      </c>
+      <c r="G12" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="H12" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="I12" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="J12" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="G12" s="19" t="s">
+      <c r="K12" s="20" t="s">
         <v>84</v>
-      </c>
-      <c r="H12" s="20" t="s">
-        <v>85</v>
-      </c>
-      <c r="I12" s="20" t="s">
-        <v>86</v>
-      </c>
-      <c r="J12" s="20" t="s">
-        <v>87</v>
-      </c>
-      <c r="K12" s="20" t="s">
-        <v>88</v>
       </c>
       <c r="L12" s="20" t="s">
         <v>20</v>
       </c>
       <c r="M12" s="20" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="N12" s="22" t="s">
         <v>49</v>
       </c>
       <c r="O12" s="23" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="P12" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="Q12" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not measured for March–August 2026. Evenor-Tech confirms no irrigation electricity-consumption measurements per hectare. Water-footprint calculations cannot supply kWh/ha. Required: dated electricity readings and irrigated area for the same farms/crops and seasonal or annual baseline. Source: Evenor-Tech confirmation, 21 October 2026. Hybrid (AMT + API) was accepted on 2 September 2026. Per-indicator routing and technical integration remain pending; auto_accept is unassigned (blank).</t>
-        </is>
+        <v>87</v>
+      </c>
+      <c r="Q12" s="20" t="s">
+        <v>115</v>
       </c>
       <c r="R12" s="30"/>
     </row>
-    <row r="13" spans="1:28" s="4" customFormat="1" ht="396.0" x14ac:dyDescent="0.2" customHeight="1">
+    <row r="13" spans="1:28" s="4" customFormat="1" ht="251.25" customHeight="1">
       <c r="A13" s="19" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="20" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="C13" s="28" t="s">
         <v>31</v>
@@ -1683,28 +1679,22 @@
       <c r="D13" s="27"/>
       <c r="E13" s="27"/>
       <c r="F13" s="24" t="s">
-        <v>94</v>
-      </c>
-      <c r="G13" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Three retained PostHog CSVs and Evenor-Tech confirmation (21 October 2026); separate read-only MongoDB aggregates.</t>
-        </is>
-      </c>
-      <c r="H13" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Check exported daily values and dates. Responsible-party confirmation identifies metric aggregation and internal tests; coverage and external-user attribution remain unverified.</t>
-        </is>
+        <v>89</v>
+      </c>
+      <c r="G13" s="20" t="s">
+        <v>116</v>
+      </c>
+      <c r="H13" s="20" t="s">
+        <v>117</v>
       </c>
       <c r="I13" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="J13" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ANFORA backend, MongoDB and PostHog. No RURACTIVE indicator feed verified.</t>
-        </is>
+      <c r="J13" s="20" t="s">
+        <v>118</v>
       </c>
       <c r="K13" s="20" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="L13" s="20" t="s">
         <v>20</v>
@@ -1716,28 +1706,22 @@
         <v>49</v>
       </c>
       <c r="O13" s="25" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="P13" s="20" t="s">
-        <v>100</v>
-      </c>
-      <c r="Q13" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1 March–31 August 2026: external users/sessions are not verified. Three PostHog CSVs show activity only on 31 August: 1 identity, 4 sessions with Pageview and 39 pageviews, as identified by the project lead, who confirms they were his own internal tests. CSVs omit query settings; full-period capture coverage is unproven. Do not infer zero external visits. Two anonymous MongoDB calculations remain separately unclassified. Sources: three retained PostHog exports and Evenor-Tech confirmation, 21 October. Hybrid (AMT + API) agreed 2 September; per-code routing, technical integration and auto_accept remain pending (blank).
-Post-monitoring developments (September–October 2026)
-Excluded from the official period. Read-only MongoDB snapshot: 21 October 2026, 12:55 CEST (Europe/Madrid). Counts by stored dates, not immutable evidence of human activity. Order: accounts / calculations / saved recipes / menus. September: 0 / 3 / 1 / 0; October to the snapshot: 28 / 55 / 27 / 3; historical totals: 33 / 60 / 28 / 3.
-Of October’s 28 accounts, 27 dated 5 October are declared by the project lead to be ADA ITS students’ personal registrations; 1 dated 21 October has unverified origin. Within the 27, 22 IDs and exact correction timestamps match the historical generator; 3 use .test domains. The declared student cohort is retained without automatically excluding 22. The provenance conflict remains unresolved; unique people are not independently verified.
-Records dated 5 October: 48 calculations, 25 recipes and 3 menus. Generator fingerprints identify 40 calculations, 22 recipes and 2 menus. Of these recipes, 20 link to declared student accounts and 2 have unresolved owners; both menus link to declared student accounts. Outside those fingerprints, 2 recipes link to one declared student account; 1 recipe and 1 menu link to an earlier account. The other 8 calculations are anonymous. Account links do not verify student authorship; unmatched records are not automatically external activity. Sources: retained aggregate reconciliation, historical generator 664e303 and responsible-party declaration. No September–October PostHog or verified session totals are available.</t>
-        </is>
+        <v>92</v>
+      </c>
+      <c r="Q13" s="20" t="s">
+        <v>134</v>
       </c>
       <c r="R13" s="30"/>
     </row>
-    <row r="14" spans="1:28" s="4" customFormat="1" ht="102.0" x14ac:dyDescent="0.2" customHeight="1">
+    <row r="14" spans="1:28" s="4" customFormat="1" ht="135" customHeight="1">
       <c r="A14" s="19" t="s">
         <v>19</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="C14" s="20" t="s">
         <v>33</v>
@@ -1745,34 +1729,28 @@
       <c r="D14" s="20"/>
       <c r="E14" s="20"/>
       <c r="F14" s="20" t="s">
-        <v>103</v>
-      </c>
-      <c r="G14" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Matched baseline and follow-up scenarios; no validated longitudinal dataset available.</t>
-        </is>
-      </c>
-      <c r="H14" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Comparable scenario analysis with consistent sources, quantities and servings.</t>
-        </is>
+        <v>94</v>
+      </c>
+      <c r="G14" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="H14" s="20" t="s">
+        <v>120</v>
       </c>
       <c r="I14" s="20" t="s">
-        <v>106</v>
-      </c>
-      <c r="J14" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Recipe footprint calculations; no verified AI recommender or behavioural-savings feed.</t>
-        </is>
+        <v>95</v>
+      </c>
+      <c r="J14" s="20" t="s">
+        <v>121</v>
       </c>
       <c r="K14" s="20" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="L14" s="20" t="s">
         <v>20</v>
       </c>
       <c r="M14" s="20" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="N14" s="22" t="s">
         <v>49</v>
@@ -1781,21 +1759,19 @@
         <v>50</v>
       </c>
       <c r="P14" s="20" t="s">
-        <v>110</v>
-      </c>
-      <c r="Q14" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not measured for March–August 2026. ANFORA supports water-footprint simulations, but no dated valid baseline/alternative scenario pairs are verified. Global versus Andalusian reference values do not establish supermarket versus local-market origin. Comparable sources, quantities and servings are required before reporting litres or percentage savings. Source: retained model/data review and Evenor-Tech confirmation, 21 October 2026. Hybrid (AMT + API) was accepted on 2 September 2026. Per-indicator routing and technical integration remain pending; auto_accept is unassigned (blank).</t>
-        </is>
+        <v>98</v>
+      </c>
+      <c r="Q14" s="20" t="s">
+        <v>122</v>
       </c>
       <c r="R14" s="30"/>
     </row>
-    <row r="15" spans="1:28" s="4" customFormat="1" ht="136.0" x14ac:dyDescent="0.2" customHeight="1">
+    <row r="15" spans="1:28" s="4" customFormat="1" ht="135.94999999999999" customHeight="1">
       <c r="A15" s="19" t="s">
         <v>19</v>
       </c>
       <c r="B15" s="20" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="C15" s="20" t="s">
         <v>34</v>
@@ -1803,57 +1779,49 @@
       <c r="D15" s="20"/>
       <c r="E15" s="20"/>
       <c r="F15" s="20" t="s">
-        <v>113</v>
-      </c>
-      <c r="G15" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Evenor-Tech confirms no numerical satisfaction survey in March-August 2026.</t>
-        </is>
-      </c>
-      <c r="H15" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No numerical cohort available; satisfaction/alert not assessable, not zero or FALSE.</t>
-        </is>
+        <v>100</v>
+      </c>
+      <c r="G15" s="20" t="s">
+        <v>123</v>
+      </c>
+      <c r="H15" s="20" t="s">
+        <v>124</v>
       </c>
       <c r="I15" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="J15" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No validated numerical survey dataset or automated alert result available.</t>
-        </is>
+        <v>101</v>
+      </c>
+      <c r="J15" s="20" t="s">
+        <v>125</v>
       </c>
       <c r="K15" s="20" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="L15" s="20" t="s">
         <v>20</v>
       </c>
       <c r="M15" s="20" t="s">
-        <v>119</v>
+        <v>103</v>
       </c>
       <c r="N15" s="26" t="s">
         <v>49</v>
       </c>
       <c r="O15" s="23" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="P15" s="20" t="s">
-        <v>121</v>
-      </c>
-      <c r="Q15" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not assessable for March–August 2026. Evenor-Tech confirms that no numerical satisfaction surveys were conducted. Neither satisfaction percentage/mean score nor the alert state can be calculated. Missing survey data do not mean a zero score or a FALSE alert. The official &lt;80% or &lt;4/5 threshold is unchanged. Source: Evenor-Tech confirmation, 21 October 2026. Hybrid (AMT + API) was accepted on 2 September 2026. Per-indicator routing and technical integration remain pending; auto_accept is unassigned (blank).</t>
-        </is>
+        <v>105</v>
+      </c>
+      <c r="Q15" s="20" t="s">
+        <v>126</v>
       </c>
       <c r="R15" s="30"/>
     </row>
-    <row r="16" spans="1:28" s="4" customFormat="1" ht="204.0" x14ac:dyDescent="0.2" customHeight="1">
+    <row r="16" spans="1:28" s="4" customFormat="1" ht="204" customHeight="1">
       <c r="A16" s="19" t="s">
         <v>19</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
       <c r="C16" s="20" t="s">
         <v>35</v>
@@ -1861,48 +1829,40 @@
       <c r="D16" s="20"/>
       <c r="E16" s="20"/>
       <c r="F16" s="20" t="s">
-        <v>124</v>
-      </c>
-      <c r="G16" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Consent-based age-group and employment declarations plus dated attendance records; dataset unavailable.</t>
-        </is>
-      </c>
-      <c r="H16" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Eligible group counts and cohort denominator required; no shares computed.</t>
-        </is>
+        <v>107</v>
+      </c>
+      <c r="G16" s="20" t="s">
+        <v>127</v>
+      </c>
+      <c r="H16" s="20" t="s">
+        <v>128</v>
       </c>
       <c r="I16" s="20" t="s">
-        <v>127</v>
-      </c>
-      <c r="J16" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Current User schema has no age-group or employment-status fields.</t>
-        </is>
+        <v>108</v>
+      </c>
+      <c r="J16" s="20" t="s">
+        <v>129</v>
       </c>
       <c r="K16" s="20" t="s">
-        <v>129</v>
+        <v>109</v>
       </c>
       <c r="L16" s="20" t="s">
         <v>20</v>
       </c>
       <c r="M16" s="20" t="s">
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="N16" s="26" t="s">
         <v>49</v>
       </c>
       <c r="O16" s="23" t="s">
-        <v>131</v>
+        <v>111</v>
       </c>
       <c r="P16" s="20" t="s">
-        <v>132</v>
-      </c>
-      <c r="Q16" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not assessable for March–August 2026. Evenor-Tech confirms insufficient demographic data. Group shares and the imbalance alert cannot be calculated without eligible group counts and a defined cohort denominator. Missing data do not establish 0% representation or a FALSE alert. Source: Evenor-Tech confirmation, 21 October 2026. Hybrid (AMT + API) was accepted on 2 September 2026. Per-indicator routing and technical integration remain pending; auto_accept is unassigned (blank).</t>
-        </is>
+        <v>112</v>
+      </c>
+      <c r="Q16" s="20" t="s">
+        <v>130</v>
       </c>
       <c r="R16" s="30"/>
     </row>
@@ -1921,15 +1881,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TranslatedLang xmlns="55fa6559-6548-493a-bddc-9eba090e1cd4" xsi:nil="true"/>
@@ -1940,6 +1891,15 @@
     <Notes_x002f_Comments xmlns="55fa6559-6548-493a-bddc-9eba090e1cd4" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2198,20 +2158,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31BC3476-64A0-47D6-BE4A-6D9019992DC0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F1FF519E-69C6-4A4F-9CD2-E1C454202659}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="55fa6559-6548-493a-bddc-9eba090e1cd4"/>
     <ds:schemaRef ds:uri="e07ec2dc-b44d-4cb9-bd12-5a2a513b4fbd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31BC3476-64A0-47D6-BE4A-6D9019992DC0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>